<commit_message>
Modified program to include Non pregnant selection item.
</commit_message>
<xml_diff>
--- a/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate.xlsx
+++ b/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blasar/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7746A37-3AD6-554F-8429-DB0E5BD7DF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C98B6B7-3F68-4A44-9944-17BB0BC42794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="V0mH21jSP57WeMvfm2GZf/CFapX9PbyX3c7CLbaowv65HEOfZYZks22oton1PO1KhMKfP/Yy+b48PowhVvmdMw==" workbookSaltValue="7RYukLmSAngqyTzJhGnEpg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="5700" yWindow="2280" windowWidth="29260" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5720" yWindow="920" windowWidth="30600" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ClinProcessing Entry Template" sheetId="6" r:id="rId1"/>
@@ -19,6 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ClinProcessing Entry Template'!$A$80:$J$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Drop-down lists'!$G$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="125">
   <si>
     <t>Id</t>
   </si>
@@ -410,6 +411,9 @@
   </si>
   <si>
     <t>Applies to Preg column with "No" value</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -894,7 +898,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J581"/>
+  <dimension ref="A1:J720"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="12" customWidth="1"/>
@@ -3638,56 +3642,473 @@
       <c r="A569" s="9"/>
       <c r="E569" s="8"/>
     </row>
+    <row r="570" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H570" s="7"/>
+    </row>
     <row r="571" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H571" s="15"/>
+      <c r="H571" s="7"/>
       <c r="I571" s="15"/>
     </row>
     <row r="572" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H572" s="15"/>
+      <c r="H572" s="7"/>
       <c r="I572" s="15"/>
     </row>
     <row r="573" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H573" s="15"/>
+      <c r="H573" s="7"/>
       <c r="I573" s="15"/>
     </row>
     <row r="574" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H574" s="15"/>
+      <c r="H574" s="7"/>
       <c r="I574" s="15"/>
     </row>
     <row r="575" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H575" s="15"/>
+      <c r="H575" s="7"/>
       <c r="I575" s="15"/>
     </row>
     <row r="576" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="H576" s="15"/>
+      <c r="H576" s="7"/>
       <c r="I576" s="15"/>
     </row>
     <row r="577" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H577" s="15"/>
+      <c r="H577" s="7"/>
       <c r="I577" s="15"/>
     </row>
     <row r="578" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H578" s="15"/>
+      <c r="H578" s="7"/>
       <c r="I578" s="15"/>
     </row>
     <row r="579" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H579" s="15"/>
+      <c r="H579" s="7"/>
       <c r="I579" s="15"/>
     </row>
     <row r="580" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H580" s="15"/>
+      <c r="H580" s="7"/>
       <c r="I580" s="15"/>
     </row>
     <row r="581" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H581" s="15"/>
+      <c r="H581" s="7"/>
       <c r="I581" s="15"/>
+    </row>
+    <row r="582" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H582" s="7"/>
+    </row>
+    <row r="583" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H583" s="7"/>
+    </row>
+    <row r="584" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H584" s="7"/>
+    </row>
+    <row r="585" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H585" s="7"/>
+    </row>
+    <row r="586" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H586" s="7"/>
+    </row>
+    <row r="587" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H587" s="7"/>
+    </row>
+    <row r="588" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H588" s="7"/>
+    </row>
+    <row r="589" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H589" s="7"/>
+    </row>
+    <row r="590" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H590" s="7"/>
+    </row>
+    <row r="591" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H591" s="7"/>
+    </row>
+    <row r="592" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H592" s="7"/>
+    </row>
+    <row r="593" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H593" s="7"/>
+    </row>
+    <row r="594" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H594" s="7"/>
+    </row>
+    <row r="595" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H595" s="7"/>
+    </row>
+    <row r="596" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H596" s="7"/>
+    </row>
+    <row r="597" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H597" s="7"/>
+    </row>
+    <row r="598" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H598" s="7"/>
+    </row>
+    <row r="599" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H599" s="7"/>
+    </row>
+    <row r="600" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H600" s="7"/>
+    </row>
+    <row r="601" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H601" s="7"/>
+    </row>
+    <row r="602" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H602" s="7"/>
+    </row>
+    <row r="603" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H603" s="7"/>
+    </row>
+    <row r="604" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H604" s="7"/>
+    </row>
+    <row r="605" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H605" s="7"/>
+    </row>
+    <row r="606" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H606" s="7"/>
+    </row>
+    <row r="607" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H607" s="7"/>
+    </row>
+    <row r="608" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H608" s="7"/>
+    </row>
+    <row r="609" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H609" s="7"/>
+    </row>
+    <row r="610" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H610" s="7"/>
+    </row>
+    <row r="611" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H611" s="7"/>
+    </row>
+    <row r="612" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H612" s="7"/>
+    </row>
+    <row r="613" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H613" s="7"/>
+    </row>
+    <row r="614" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H614" s="7"/>
+    </row>
+    <row r="615" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H615" s="7"/>
+    </row>
+    <row r="616" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H616" s="7"/>
+    </row>
+    <row r="617" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H617" s="7"/>
+    </row>
+    <row r="618" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H618" s="7"/>
+    </row>
+    <row r="619" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H619" s="7"/>
+    </row>
+    <row r="620" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H620" s="7"/>
+    </row>
+    <row r="621" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H621" s="7"/>
+    </row>
+    <row r="622" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H622" s="7"/>
+    </row>
+    <row r="623" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H623" s="7"/>
+    </row>
+    <row r="624" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H624" s="7"/>
+    </row>
+    <row r="625" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H625" s="7"/>
+    </row>
+    <row r="626" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H626" s="7"/>
+    </row>
+    <row r="627" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H627" s="7"/>
+    </row>
+    <row r="628" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H628" s="7"/>
+    </row>
+    <row r="629" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H629" s="7"/>
+    </row>
+    <row r="630" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H630" s="7"/>
+    </row>
+    <row r="631" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H631" s="7"/>
+    </row>
+    <row r="632" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H632" s="7"/>
+    </row>
+    <row r="633" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H633" s="7"/>
+    </row>
+    <row r="634" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H634" s="7"/>
+    </row>
+    <row r="635" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H635" s="7"/>
+    </row>
+    <row r="636" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H636" s="7"/>
+    </row>
+    <row r="637" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H637" s="7"/>
+    </row>
+    <row r="638" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H638" s="7"/>
+    </row>
+    <row r="639" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H639" s="7"/>
+    </row>
+    <row r="640" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H640" s="7"/>
+    </row>
+    <row r="641" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H641" s="7"/>
+    </row>
+    <row r="642" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H642" s="7"/>
+    </row>
+    <row r="643" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H643" s="7"/>
+    </row>
+    <row r="644" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H644" s="7"/>
+    </row>
+    <row r="645" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H645" s="7"/>
+    </row>
+    <row r="646" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H646" s="7"/>
+    </row>
+    <row r="647" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H647" s="7"/>
+    </row>
+    <row r="648" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H648" s="7"/>
+    </row>
+    <row r="649" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H649" s="7"/>
+    </row>
+    <row r="650" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H650" s="7"/>
+    </row>
+    <row r="651" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H651" s="7"/>
+    </row>
+    <row r="652" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H652" s="7"/>
+    </row>
+    <row r="653" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H653" s="7"/>
+    </row>
+    <row r="654" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H654" s="7"/>
+    </row>
+    <row r="655" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H655" s="7"/>
+    </row>
+    <row r="656" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H656" s="7"/>
+    </row>
+    <row r="657" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H657" s="7"/>
+    </row>
+    <row r="658" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H658" s="7"/>
+    </row>
+    <row r="659" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H659" s="7"/>
+    </row>
+    <row r="660" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H660" s="7"/>
+    </row>
+    <row r="661" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H661" s="7"/>
+    </row>
+    <row r="662" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H662" s="7"/>
+    </row>
+    <row r="663" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H663" s="7"/>
+    </row>
+    <row r="664" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H664" s="7"/>
+    </row>
+    <row r="665" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H665" s="7"/>
+    </row>
+    <row r="666" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H666" s="7"/>
+    </row>
+    <row r="667" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H667" s="7"/>
+    </row>
+    <row r="668" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H668" s="7"/>
+    </row>
+    <row r="669" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H669" s="7"/>
+    </row>
+    <row r="670" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H670" s="7"/>
+    </row>
+    <row r="671" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H671" s="7"/>
+    </row>
+    <row r="672" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H672" s="7"/>
+    </row>
+    <row r="673" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H673" s="7"/>
+    </row>
+    <row r="674" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H674" s="7"/>
+    </row>
+    <row r="675" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H675" s="7"/>
+    </row>
+    <row r="676" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H676" s="7"/>
+    </row>
+    <row r="677" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H677" s="7"/>
+    </row>
+    <row r="678" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H678" s="7"/>
+    </row>
+    <row r="679" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H679" s="7"/>
+    </row>
+    <row r="680" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H680" s="7"/>
+    </row>
+    <row r="681" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H681" s="7"/>
+    </row>
+    <row r="682" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H682" s="7"/>
+    </row>
+    <row r="683" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H683" s="7"/>
+    </row>
+    <row r="684" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H684" s="7"/>
+    </row>
+    <row r="685" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H685" s="7"/>
+    </row>
+    <row r="686" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H686" s="7"/>
+    </row>
+    <row r="687" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H687" s="7"/>
+    </row>
+    <row r="688" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H688" s="7"/>
+    </row>
+    <row r="689" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H689" s="7"/>
+    </row>
+    <row r="690" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H690" s="7"/>
+    </row>
+    <row r="691" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H691" s="7"/>
+    </row>
+    <row r="692" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H692" s="7"/>
+    </row>
+    <row r="693" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H693" s="7"/>
+    </row>
+    <row r="694" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H694" s="7"/>
+    </row>
+    <row r="695" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H695" s="7"/>
+    </row>
+    <row r="696" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H696" s="7"/>
+    </row>
+    <row r="697" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H697" s="7"/>
+    </row>
+    <row r="698" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H698" s="7"/>
+    </row>
+    <row r="699" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H699" s="7"/>
+    </row>
+    <row r="700" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H700" s="7"/>
+    </row>
+    <row r="701" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H701" s="7"/>
+    </row>
+    <row r="702" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H702" s="7"/>
+    </row>
+    <row r="703" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H703" s="7"/>
+    </row>
+    <row r="704" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H704" s="7"/>
+    </row>
+    <row r="705" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H705" s="7"/>
+    </row>
+    <row r="706" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H706" s="7"/>
+    </row>
+    <row r="707" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H707" s="7"/>
+    </row>
+    <row r="708" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H708" s="7"/>
+    </row>
+    <row r="710" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H710" s="15"/>
+    </row>
+    <row r="711" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H711" s="15"/>
+    </row>
+    <row r="712" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H712" s="15"/>
+    </row>
+    <row r="713" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H713" s="15"/>
+    </row>
+    <row r="714" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H714" s="15"/>
+    </row>
+    <row r="715" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H715" s="15"/>
+    </row>
+    <row r="716" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H716" s="15"/>
+    </row>
+    <row r="717" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H717" s="15"/>
+    </row>
+    <row r="718" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H718" s="15"/>
+    </row>
+    <row r="719" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H719" s="15"/>
+    </row>
+    <row r="720" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H720" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
           <x14:formula1>
             <xm:f>'Drop-down lists'!#REF!</xm:f>
@@ -3718,17 +4139,23 @@
           </x14:formula1>
           <xm:sqref>G69:G569</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
-          <x14:formula1>
-            <xm:f>'Drop-down lists'!$G$2:$G$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>H69:H569</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000006000000}">
           <x14:formula1>
             <xm:f>'Drop-down lists'!$H$2:$H$3</xm:f>
           </x14:formula1>
           <xm:sqref>I69:I569</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
+          <x14:formula1>
+            <xm:f>'Drop-down lists'!$G$2:$G$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>H69 H209:H708</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25E1E495-68A7-8D49-B0E7-753B3990CBA7}">
+          <x14:formula1>
+            <xm:f>'Drop-down lists'!$G$2:$G$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>H70:H208</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3848,7 +4275,9 @@
         <v>3</v>
       </c>
       <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3" t="s">
+        <v>124</v>
+      </c>
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Modified Clinical upload template.
</commit_message>
<xml_diff>
--- a/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate.xlsx
+++ b/onprc_ehr/resources/web/onprc_ehr/templates/ClinicalProcessingTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blasar/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C98B6B7-3F68-4A44-9944-17BB0BC42794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4B6F4B-8562-3946-A936-D3ECBBD18399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="V0mH21jSP57WeMvfm2GZf/CFapX9PbyX3c7CLbaowv65HEOfZYZks22oton1PO1KhMKfP/Yy+b48PowhVvmdMw==" workbookSaltValue="7RYukLmSAngqyTzJhGnEpg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="5720" yWindow="920" windowWidth="30600" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -1599,12 +1599,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="13"/>
       <c r="B67" s="3"/>
       <c r="D67" s="15"/>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="13" t="s">
         <v>0</v>
       </c>
@@ -4155,7 +4155,7 @@
           <x14:formula1>
             <xm:f>'Drop-down lists'!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>H70:H208</xm:sqref>
+          <xm:sqref>H167:H208 H70:H166</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>